<commit_message>
Dados atualizados via robô v2
</commit_message>
<xml_diff>
--- a/sipii_caixa_20260515.xlsx
+++ b/sipii_caixa_20260515.xlsx
@@ -899,7 +899,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>409,139</t>
+          <t>407,507</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>6.692,462</t>
+          <t>6.642,127</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>821,940</t>
+          <t>809,364</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>120,061</t>
+          <t>120,060</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>96,154</t>
+          <t>96,103</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>584,815</t>
+          <t>584,810</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>61,661</t>
+          <t>61,659</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>1.674,048</t>
+          <t>1.674,014</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -4019,7 +4019,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>28,460</t>
+          <t>28,459</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -4963,7 +4963,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>79,762</t>
+          <t>79,748</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>141,198</t>
+          <t>141,196</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -6216,7 +6216,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1.749,908</t>
+          <t>1.739,994</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -6520,7 +6520,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2.197,946</t>
+          <t>2.197,935</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -6834,7 +6834,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>13,221</t>
+          <t>13,218</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -7459,7 +7459,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>956,924</t>
+          <t>956,919</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -7739,7 +7739,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT ARX IPCA DEB INCENTIVADAS FIC FIF RF CRED PRIV - RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT ARX IPCA DEB INCENTIVADAS FIC FIF RF CRED PRIV - RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -7749,32 +7749,32 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,10822667</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>-0,16</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>2,73</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>219,275</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -8038,7 +8038,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF FIC EXPERT SULAMERICA RF CRED PRIV LP - RESP LTDA (1)</t>
+          <t>CAIXA FIF FIC EXPERT SULAMERICA RF CRED PRIV LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -8048,32 +8048,32 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,22725900</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>0,55</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>4,78</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>14,62</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>70,959</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>175,201</t>
+          <t>175,171</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -8944,7 +8944,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT VOX DESENV SUSTENTAVEL IS RF CRED PRIV LP - RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT VOX DESENV SUSTENTAVEL IS RF CRED PRIV LP - RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -8954,32 +8954,32 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,02873200</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>0,46</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>4,91</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>21,741</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -9226,7 +9226,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT ABSOLUTE CRETA FIC FIF RF CRED PRIV LP - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT ABSOLUTE CRETA FIC FIF RF CRED PRIV LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -9236,32 +9236,32 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,15477900</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>0,57</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>3,99</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>13,71</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>66,609</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -9524,7 +9524,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT RB ASSET CDI DEB INCENTIVADAS FIC FIF RF CRED PRIV RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT RB ASSET CDI DEB INCENTIVADAS FIC FIF RF CRED PRIV RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -9534,32 +9534,32 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,05746535</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>0,28</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>2,33</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>333,972</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT VINLAND DEB IN INFRA RF CRED PRIV LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA EXPERT VINLAND DEB IN INFRA RF CRED PRIV LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -10142,7 +10142,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>859,794</t>
+          <t>859,244</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -10448,7 +10448,7 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>3.239,969</t>
+          <t>3.239,895</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>3.112,250</t>
+          <t>3.112,204</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -11373,7 +11373,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>125,190</t>
+          <t>125,111</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -11675,7 +11675,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>546,370</t>
+          <t>546,362</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -12306,7 +12306,7 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>333,818</t>
+          <t>333,813</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -12612,7 +12612,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>2.373,986</t>
+          <t>2.373,977</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -13239,7 +13239,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>15.478,842</t>
+          <t>15.478,557</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -13560,7 +13560,7 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>1.382,856</t>
+          <t>1.382,850</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -13872,7 +13872,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>165,448</t>
+          <t>165,441</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -14467,7 +14467,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>5.993,518</t>
+          <t>5.939,950</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -14775,7 +14775,7 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>2.187,961</t>
+          <t>2.187,914</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -15413,7 +15413,7 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>840,007</t>
+          <t>840,001</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
@@ -15732,7 +15732,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>15.529,915</t>
+          <t>15.529,642</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -16022,7 +16022,7 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>9.455,244</t>
+          <t>9.456,377</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -16340,7 +16340,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>20.820,632</t>
+          <t>20.820,212</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -16663,7 +16663,7 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>13.120,421</t>
+          <t>13.120,302</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
@@ -16986,7 +16986,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>251,344</t>
+          <t>251,355</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -17258,7 +17258,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART CRED PRIV MM LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART CRED PRIV MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -17268,32 +17268,32 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,39942200</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,000</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>0,61</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>4,52</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>14,20</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>68,867</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC MULTIGESTOR GLOBAL EQUITIES IE (1)</t>
+          <t>CAIXA FIC MULTIGESTOR GLOBAL EQUITIES IE</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -17562,32 +17562,32 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.167,28992200</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>1,55</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>-6,97</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>-1,30</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>35,740</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>329,516</t>
+          <t>540,035</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ESTRATÉGIA LIVRE MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF ESTRATÉGIA LIVRE MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -18000,32 +18000,32 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.628,88339000</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>-0,006</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>-0,42</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>3,95</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>13,25</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>117,176</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -18598,7 +18598,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT DUO FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT DUO FIC FIF MM LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -18884,7 +18884,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART LONG SHORT LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART LONG SHORT LP RESP LTDA</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -18894,32 +18894,32 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,24727900</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>-0,67</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>2,12</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>11,59</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6,651</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -19500,7 +19500,7 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT QUALI FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT QUALI FIC FIF MM LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -19786,7 +19786,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART LONG BIAS MM RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART LONG BIAS MM RESP LTDA</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -19796,32 +19796,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,43731600</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>-2,13</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>5,29</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>21,02</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12,206</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -20088,7 +20088,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT UNO FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT UNO FIC FIF MM LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -20409,7 +20409,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>3,162</t>
+          <t>3,160</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -20696,7 +20696,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ESTRATÉGICO MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF ESTRATÉGICO MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -20706,32 +20706,32 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>5,31164077</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>-0,37</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>3,51</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>13,01</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>33,135</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
@@ -21045,7 +21045,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>686,347</t>
+          <t>685,158</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -21320,7 +21320,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART MULTIESTRATEGIA MM RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART MULTIESTRATEGIA MM RESP LTDA</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -21330,32 +21330,32 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>2,84815900</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>-0,16</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>1,97</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>11,32</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>77,176</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -21661,7 +21661,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>31,999</t>
+          <t>31,981</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -21971,7 +21971,7 @@
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>2.357,364</t>
+          <t>2.357,295</t>
         </is>
       </c>
       <c r="J71" s="4" t="inlineStr">
@@ -22556,7 +22556,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FUNCIONARIOS ESTRATEGIA LIVRE MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FUNCIONARIOS ESTRATEGIA LIVRE MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -22566,32 +22566,32 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.649,20997000</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>-0,38</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>4,28</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>14,21</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>15,281</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
@@ -22842,7 +22842,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>CAIXA HASHDEX NASDAQ CRYPTO INDEX FIC FIF MM RESP LTDA (1) (2)</t>
+          <t>CAIXA HASHDEX NASDAQ CRYPTO INDEX FIC FIF MM RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -22852,32 +22852,32 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,56381485</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>-0,007</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>3,92</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>-21,91</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4,109</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF CAPITAL PROTEGIDO CESTA AGRO MM (1)</t>
+          <t>CAIXA FIC FIF CAPITAL PROTEGIDO CESTA AGRO MM</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -23161,32 +23161,32 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,38641800</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>-0,80</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>2,23</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>9,04</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>71,165</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
@@ -23472,7 +23472,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC FIF MM LP - RESP LTDA (1)</t>
+          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC FIF MM LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -23482,32 +23482,32 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,53122700</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>-0,14</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>2,55</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>19,20</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14,493</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -23792,7 +23792,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL PROTEGIDO IBOVESPA CÍCLICO I FIC FIF MM (1)</t>
+          <t>CAIXA CAPITAL PROTEGIDO IBOVESPA CÍCLICO I FIC FIF MM</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -23802,32 +23802,32 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>3,24198200</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>0,75</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>1,75</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>7,27</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>154,478</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
@@ -24108,7 +24108,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIM CAPITAL PROTEGIDO CICLICO II LP - RL (1)</t>
+          <t>CAIXA FIC FIM CAPITAL PROTEGIDO CICLICO II LP - RL</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -24118,32 +24118,32 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,47354200</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>1,60</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>1,89</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>14,51</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>191,149</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -24429,7 +24429,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EXPERT PIMCO INCOME IE MM LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF EXPERT PIMCO INCOME IE MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -24439,32 +24439,32 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,41225500</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>0,26</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>16,57</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>279,225</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
@@ -24740,7 +24740,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT GIANT ZARATHUSTRA FIC MULTIMERCADO - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT GIANT ZARATHUSTRA FIC MULTIMERCADO - RESP LTDA</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -24750,32 +24750,32 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,31342200</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>0,32</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>2,33</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>2,77</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13,409</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -25086,7 +25086,7 @@
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>899,737</t>
+          <t>899,702</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
@@ -25408,7 +25408,7 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>750,502</t>
+          <t>750,501</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -25683,7 +25683,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>FIC FIF CAIXA EXPERT BTG PACTUAL X10 MM LP RESP LTDA (1)</t>
+          <t>FIC FIF CAIXA EXPERT BTG PACTUAL X10 MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -25693,32 +25693,32 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>6,77440300</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>-0,05</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>5,33</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>16,66</t>
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>129,413</t>
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr">
@@ -25990,7 +25990,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EXPERT SPX NIMITZ MULTIMERCADO RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF EXPERT SPX NIMITZ MULTIMERCADO RESP LTDA</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -26000,32 +26000,32 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,77044700</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>0,62</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>0,22</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>10,26</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>176,345</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -26328,7 +26328,7 @@
       </c>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>96,091</t>
+          <t>96,085</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr">
@@ -26638,7 +26638,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>349,198</t>
+          <t>349,196</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -27557,7 +27557,7 @@
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>277,785</t>
+          <t>277,682</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr">
@@ -27867,7 +27867,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>452,035</t>
+          <t>451,985</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -28185,7 +28185,7 @@
       </c>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>58,805</t>
+          <t>58,800</t>
         </is>
       </c>
       <c r="J91" s="4" t="inlineStr">
@@ -28499,7 +28499,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>2,322</t>
+          <t>2,312</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -28819,7 +28819,7 @@
       </c>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>81,498</t>
+          <t>81,393</t>
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr">
@@ -29129,7 +29129,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>92,847</t>
+          <t>92,821</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -29408,7 +29408,7 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF AÇÕES MULTIGESTOR RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF AÇÕES MULTIGESTOR RESP LTDA</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -29418,32 +29418,32 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,28913400</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>-0,022</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>-5,59</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>0,15</t>
+        </is>
+      </c>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>10,68</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>292,745</t>
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr">
@@ -29753,7 +29753,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>116,457</t>
+          <t>116,342</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -30385,7 +30385,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>48,277</t>
+          <t>48,276</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -30703,7 +30703,7 @@
       </c>
       <c r="I99" s="4" t="inlineStr">
         <is>
-          <t>128,524</t>
+          <t>128,522</t>
         </is>
       </c>
       <c r="J99" s="4" t="inlineStr">
@@ -31021,7 +31021,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>41,059</t>
+          <t>40,986</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -31327,7 +31327,7 @@
       </c>
       <c r="I101" s="4" t="inlineStr">
         <is>
-          <t>673,018</t>
+          <t>672,434</t>
         </is>
       </c>
       <c r="J101" s="4" t="inlineStr">
@@ -31645,7 +31645,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>444,214</t>
+          <t>444,047</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -32886,7 +32886,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>44,644</t>
+          <t>44,632</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -33184,7 +33184,7 @@
       </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
-          <t>36,555</t>
+          <t>36,528</t>
         </is>
       </c>
       <c r="J107" s="4" t="inlineStr">
@@ -33498,7 +33498,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>890,836</t>
+          <t>890,306</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -33816,7 +33816,7 @@
       </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
-          <t>3,036</t>
+          <t>3,035</t>
         </is>
       </c>
       <c r="J109" s="4" t="inlineStr">
@@ -34730,7 +34730,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>273,319</t>
+          <t>273,034</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -35009,7 +35009,7 @@
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC ACOES EXPERT VERDE AM LONG BIAS - RESP LTDA (1)</t>
+          <t>CAIXA FIC ACOES EXPERT VERDE AM LONG BIAS - RESP LTDA</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
@@ -35019,32 +35019,32 @@
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.010,65879200</t>
+        </is>
+      </c>
+      <c r="E113" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>-5,54</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>3,09</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>18,98</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8,117</t>
         </is>
       </c>
       <c r="J113" s="4" t="inlineStr">
@@ -35324,7 +35324,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT CLARITAS VALOR FIC FIF AÇÕES - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT CLARITAS VALOR FIC FIF AÇÕES - RESP LTDA</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -35334,32 +35334,32 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.523,08345000</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F114" s="7" t="inlineStr">
+        <is>
+          <t>-5,32</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>1,82</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>15,16</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22,184</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -35641,7 +35641,7 @@
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>174,02337300</t>
+          <t>174,02337331</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
@@ -36087,7 +36087,7 @@
       </c>
       <c r="I117" s="4" t="inlineStr">
         <is>
-          <t>1.713,567</t>
+          <t>1.713,039</t>
         </is>
       </c>
       <c r="J117" s="4" t="inlineStr">
@@ -36386,7 +36386,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>716,044</t>
+          <t>715,521</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -36672,7 +36672,7 @@
       </c>
       <c r="I119" s="4" t="inlineStr">
         <is>
-          <t>791,357</t>
+          <t>791,211</t>
         </is>
       </c>
       <c r="J119" s="4" t="inlineStr">
@@ -36962,7 +36962,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>115,860</t>
+          <t>115,871</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -37552,7 +37552,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>620,469</t>
+          <t>620,064</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -37843,7 +37843,7 @@
       </c>
       <c r="I123" s="4" t="inlineStr">
         <is>
-          <t>473,892</t>
+          <t>473,802</t>
         </is>
       </c>
       <c r="J123" s="4" t="inlineStr">
@@ -38133,7 +38133,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>713,997</t>
+          <t>713,106</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -38716,7 +38716,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>283,611</t>
+          <t>278,180</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -40277,7 +40277,7 @@
       </c>
       <c r="I131" s="4" t="inlineStr">
         <is>
-          <t>7.890,362</t>
+          <t>7.735,561</t>
         </is>
       </c>
       <c r="J131" s="4" t="inlineStr">
@@ -40586,7 +40586,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>15.080,332</t>
+          <t>15.080,057</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -40895,7 +40895,7 @@
       </c>
       <c r="I133" s="4" t="inlineStr">
         <is>
-          <t>3.135,259</t>
+          <t>3.135,214</t>
         </is>
       </c>
       <c r="J133" s="4" t="inlineStr">
@@ -41187,7 +41187,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>1,53751100</t>
+          <t>1,53751081</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
@@ -41801,7 +41801,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>3.987,907</t>
+          <t>3.987,906</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -42398,7 +42398,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>13.511,514</t>
+          <t>13.316,841</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -42707,7 +42707,7 @@
       </c>
       <c r="I139" s="4" t="inlineStr">
         <is>
-          <t>12.285,698</t>
+          <t>12.285,686</t>
         </is>
       </c>
       <c r="J139" s="4" t="inlineStr">
@@ -43029,7 +43029,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>3.879,486</t>
+          <t>3.879,335</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -43648,7 +43648,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>32.872,839</t>
+          <t>33.519,553</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -43955,7 +43955,7 @@
       </c>
       <c r="I143" s="4" t="inlineStr">
         <is>
-          <t>2.841,802</t>
+          <t>2.913,693</t>
         </is>
       </c>
       <c r="J143" s="4" t="inlineStr">
@@ -44268,7 +44268,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>14.318,538</t>
+          <t>14.472,781</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -44386,7 +44386,7 @@
       </c>
       <c r="I145" s="4" t="inlineStr">
         <is>
-          <t>9.177,447</t>
+          <t>9.177,440</t>
         </is>
       </c>
       <c r="J145" s="4" t="inlineStr">
@@ -45968,7 +45968,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>2.954,719</t>
+          <t>2.954,715</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -48507,7 +48507,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>13.150,977</t>
+          <t>13.150,970</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -49445,7 +49445,7 @@
       </c>
       <c r="I161" s="4" t="inlineStr">
         <is>
-          <t>1.489,799</t>
+          <t>1.553,865</t>
         </is>
       </c>
       <c r="J161" s="4" t="inlineStr">
@@ -49757,7 +49757,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>24.837,969</t>
+          <t>24.837,967</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -50693,7 +50693,7 @@
       </c>
       <c r="I165" s="4" t="inlineStr">
         <is>
-          <t>302,859</t>
+          <t>302,833</t>
         </is>
       </c>
       <c r="J165" s="4" t="inlineStr">
@@ -51300,7 +51300,7 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>11,25841100</t>
+          <t>11,25841071</t>
         </is>
       </c>
       <c r="E167" s="5" t="inlineStr">
@@ -52234,7 +52234,7 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>3,49647100</t>
+          <t>3,49647080</t>
         </is>
       </c>
       <c r="E170" s="3" t="inlineStr">
@@ -52544,7 +52544,7 @@
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>2,56190500</t>
+          <t>2,56190497</t>
         </is>
       </c>
       <c r="E171" s="5" t="inlineStr">
@@ -52875,7 +52875,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>5.026,537</t>
+          <t>5.026,126</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">

</xml_diff>